<commit_message>
process tweaks and clearer naming
</commit_message>
<xml_diff>
--- a/templates/xlsx/chillibyte-project-trackers.xlsx
+++ b/templates/xlsx/chillibyte-project-trackers.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gate tracker" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estimate baseline" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision log" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change log" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variation register" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sitemap" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Page inventory" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content matrix" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Block inventory" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; assumptions" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Read me" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Gate tracker" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Estimate baseline" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Decision log" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Change log" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Variation register" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Sitemap" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Page inventory" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Content matrix" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Block inventory" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Risks &amp; assumptions" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="QA" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Launch" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Gate tracker'!$A$3:$O$28</definedName>
@@ -763,7 +763,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Approved at Gate 5. Collapse duplicates hard — if this list is as long as your section list, no consolidation has happened.</t>
+          <t>Approved at the block inventory approval. Collapse duplicates hard — if this list is as long as your section list, no consolidation has happened.</t>
         </is>
       </c>
     </row>
@@ -2376,7 +2376,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Tested against the support matrix and accessibility target agreed at Gate 1 — and nothing beyond them. That is what makes QA finishable.</t>
+          <t>Tested against the support matrix and accessibility target agreed at the discovery approval — and nothing beyond them. That is what makes QA finishable.</t>
         </is>
       </c>
     </row>
@@ -3261,7 +3261,7 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Final client approval captured (Gate 12)</t>
+          <t>Final client approval captured</t>
         </is>
       </c>
       <c r="C4" s="9" t="n"/>
@@ -3272,7 +3272,7 @@
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>Gate 12</t>
+          <t>Staging approval</t>
         </is>
       </c>
       <c r="F4" s="9" t="n"/>
@@ -3299,7 +3299,7 @@
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>Gate 12</t>
+          <t>Staging approval</t>
         </is>
       </c>
       <c r="F5" s="9" t="n"/>
@@ -3457,7 +3457,7 @@
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>Gate C5</t>
+          <t>Compliance approval</t>
         </is>
       </c>
       <c r="F11" s="9" t="n"/>
@@ -3530,7 +3530,7 @@
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>Gate 13</t>
+          <t>Launch approval</t>
         </is>
       </c>
       <c r="F14" s="9" t="n"/>
@@ -3557,7 +3557,7 @@
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>Gate 13</t>
+          <t>Launch approval</t>
         </is>
       </c>
       <c r="F15" s="9" t="n"/>
@@ -3978,7 +3978,7 @@
   <dimension ref="A1:O28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
@@ -4012,7 +4012,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Gate</t>
+          <t>Approval</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
@@ -4089,12 +4089,12 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Studio brief</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Sales handover accepted</t>
+          <t>Studio brief accepted</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
@@ -4104,7 +4104,7 @@
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>Sales handover note v1.0</t>
+          <t>Studio brief v1.0</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
@@ -4119,7 +4119,7 @@
       </c>
       <c r="G4" s="8" t="inlineStr">
         <is>
-          <t>Gate 0: sales handover accepted</t>
+          <t>Approval: studio brief</t>
         </is>
       </c>
       <c r="H4" s="8" t="inlineStr">
@@ -4588,8 +4588,8 @@
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="29" customWidth="1" min="3" max="3"/>
-    <col width="33" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
@@ -4607,7 +4607,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Set at Gate 1, re-baselined at Gate 10, actuals recorded at Gate 14. Without this, scope creep cannot be demonstrated — only asserted.</t>
+          <t>Set at the discovery approval, re-baselined at the build specification approval, actuals recorded at the project closure approval. Without this, scope creep cannot be demonstrated — only asserted.</t>
         </is>
       </c>
     </row>
@@ -4624,12 +4624,12 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Gate 1 baseline (hrs)</t>
+          <t>Discovery baseline (hrs)</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>Gate 10 re-baseline (hrs)</t>
+          <t>Build spec re-baseline (hrs)</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
@@ -5223,7 +5223,7 @@
       </c>
       <c r="M4" s="8" t="inlineStr">
         <is>
-          <t>Basecamp Gate 1</t>
+          <t>Approval: discovery ticket</t>
         </is>
       </c>
       <c r="N4" s="8" t="inlineStr">
@@ -7215,7 +7215,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Approved at Gate 3. Where there is an existing site, every old URL maps to a new one or to a documented retirement.</t>
+          <t>Approved at the sitemap approval. Where there is an existing site, every old URL maps to a new one or to a documented retirement.</t>
         </is>
       </c>
     </row>

</xml_diff>